<commit_message>
Add MIT license, version table, references; re-run evaluation on final code
- MIT license (LICENSE, pyproject metadata, README section)
- README: tested versions (Python, Ollama, model digest, packages),
  `init` in the command reference, link to the schema
- Design doc and report: references and evidence-index appendices;
  timing numbers from the new run
- Evaluation harness now runs with a clean environment and ignores .env
  (CK_IGNORE_DOTENV), so personal mail settings can never reach results/
- Sample-mail generator uses a fixed MIME boundary, so regenerated
  fixtures are byte-identical
- Results regenerated on the final code: 12/12 scenarios, memory on 3/3
  vs off 0/3, 5/5 sampled claims, 0 duplicate deliveries

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/runs/main/exports/maryam_register.xlsx
+++ b/results/runs/main/exports/maryam_register.xlsx
@@ -642,7 +642,7 @@
       <c r="S2" s="3" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T20:33:33+00:00</t>
+          <t>2026-10-28T21:43:38+00:00</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Rule 3: Imran Qadir owes the commitment 'Send comments on proposal draft to Maryam Siddiqui' which is overdue (due 2026-11-04). Nudges sent: 0/2. Recent message m11.maryam@fixtures.commitkeeper claims he sent comments, but the user's confirm_completion was rejected, indicating the task remains unfulfilled.</t>
+          <t>Rule 3: Imran Qadir owes Maryam comments on the proposal draft (due 2026-11-04), which is overdue by 8 days. No nudges have been sent yet (limit 2).</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -730,7 +730,7 @@
       <c r="S3" s="3" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T20:33:33+00:00</t>
+          <t>2026-10-28T21:43:38+00:00</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Rule 2: User owes the commitment and it is due today (2026-11-02). The due date is within 1 day, so a reminder is needed.</t>
+          <t>Rule 2: User owes the commitment, and it is due today (2026-11-02). The due date is within 1 day, so a reminder is needed.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -810,7 +810,7 @@
       <c r="S4" s="3" t="inlineStr"/>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T20:33:33+00:00</t>
+          <t>2026-10-28T21:43:38+00:00</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Rule 1: Recent message m13 shows Bilal is away until 14 November (after today's date), so following up now would be premature. The commitment is overdue by 6 days, but the pending unavailability overrides rules 2-4.</t>
+          <t>Bilal's automatic reply (message 13) indicates he is away until 14 November, which is after today (12 November). Rule 1 overrides other rules, so we must wait before following up.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -894,7 +894,7 @@
       <c r="S5" s="3" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T20:33:33+00:00</t>
+          <t>2026-10-28T21:43:38+00:00</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>The user owes the assignment, which is due today (2026-11-12). The deadline was extended to today and approved by the user on 2026-11-09.</t>
+          <t>Rule 2: User owes the assignment and it is due today (2026-11-12). The due date is imminent, requiring a reminder despite the low nudge count.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -974,7 +974,7 @@
       <c r="S6" s="3" t="inlineStr"/>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T20:33:33+00:00</t>
+          <t>2026-10-28T21:43:38+00:00</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       <c r="S7" s="3" t="inlineStr"/>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T20:33:33+00:00</t>
+          <t>2026-10-28T21:43:38+00:00</t>
         </is>
       </c>
     </row>
@@ -1773,7 +1773,7 @@
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Rule 2: User owes the commitment and it is due today (2026-11-02). The due date is within 1 day, so a reminder is needed.</t>
+          <t>Rule 2: User owes the commitment, and it is due today (2026-11-02). The due date is within 1 day, so a reminder is needed.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -2093,7 +2093,7 @@
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Rule 3: Bilal owes the commitment 'Share annotated dataset with Maryam' which is overdue by 3 days. Nudges sent: 0 (limit 2).</t>
+          <t>Bilal owes the commitment 'Share annotated dataset with Maryam' which is overdue by 3 days. No nudges have been sent yet, below the 2-nudge limit.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -2155,7 +2155,7 @@
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Rule 3: Imran Qadir owes the commitment 'Send comments on proposal draft to Maryam Siddiqui' which is overdue (due 2026-11-04). Nudges sent: 0/2. Recent message m11.maryam@fixtures.commitkeeper claims he sent comments, but the user's confirm_completion was rejected, indicating the task remains unfulfilled.</t>
+          <t>Rule 3: Imran Qadir owes Maryam comments on the proposal draft (due 2026-11-04), which is overdue by 8 days. No nudges have been sent yet (limit 2).</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -2205,7 +2205,7 @@
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>The user owes the assignment, which is due today (2026-11-12). The deadline was extended to today and approved by the user on 2026-11-09.</t>
+          <t>Rule 2: User owes the assignment and it is due today (2026-11-12). The due date is imminent, requiring a reminder despite the low nudge count.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>exported 2026-10-28T20:33:33+00:00</t>
+          <t>exported 2026-10-28T21:43:38+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>